<commit_message>
Linha Body Splash Inspiração no site e catálogo atualizado
Nova seção com 25 body splashes de inspiração (selo verde), item no
menu, filtro na busca, cartão nas categorias e tabela de valores.
Fotos com fundo cinza viram brancas e a do Baby John é recortada.
Inclui o catálogo em PDF atualizado e o Guia de Experiência.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/arquivos/Fragrâncias Alquimikamente - FINAL.xlsx
+++ b/arquivos/Fragrâncias Alquimikamente - FINAL.xlsx
@@ -7,7 +7,7 @@
     <sheet name="Legenda" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Fragrâncias'!$A$1:$F$299</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Fragrâncias'!$A$1:$F$324</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -53,7 +53,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -101,6 +101,11 @@
         <fgColor rgb="00C8E6C9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BBDEFB"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border/>
@@ -128,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -151,6 +156,9 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -426,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F299"/>
+  <dimension ref="A1:F324"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="38" customWidth="1" style="16" min="1" max="1"/>
@@ -10005,31 +10013,806 @@
         </is>
       </c>
     </row>
-    <row r="300" ht="15.75" customHeight="1" s="16"/>
-    <row r="301" ht="15.75" customHeight="1" s="16"/>
-    <row r="302" ht="15.75" customHeight="1" s="16"/>
-    <row r="303" ht="15.75" customHeight="1" s="16"/>
-    <row r="304" ht="15.75" customHeight="1" s="16"/>
-    <row r="305" ht="15.75" customHeight="1" s="16"/>
-    <row r="306" ht="15.75" customHeight="1" s="16"/>
-    <row r="307" ht="15.75" customHeight="1" s="16"/>
-    <row r="308" ht="15.75" customHeight="1" s="16"/>
-    <row r="309" ht="15.75" customHeight="1" s="16"/>
-    <row r="310" ht="15.75" customHeight="1" s="16"/>
-    <row r="311" ht="15.75" customHeight="1" s="16"/>
-    <row r="312" ht="15.75" customHeight="1" s="16"/>
-    <row r="313" ht="15.75" customHeight="1" s="16"/>
-    <row r="314" ht="15.75" customHeight="1" s="16"/>
-    <row r="315" ht="15.75" customHeight="1" s="16"/>
-    <row r="316" ht="15.75" customHeight="1" s="16"/>
-    <row r="317" ht="15.75" customHeight="1" s="16"/>
-    <row r="318" ht="15.75" customHeight="1" s="16"/>
-    <row r="319" ht="15.75" customHeight="1" s="16"/>
-    <row r="320" ht="15.75" customHeight="1" s="16"/>
-    <row r="321" ht="15.75" customHeight="1" s="16"/>
-    <row r="322" ht="15.75" customHeight="1" s="16"/>
-    <row r="323" ht="15.75" customHeight="1" s="16"/>
-    <row r="324" ht="15.75" customHeight="1" s="16"/>
+    <row r="300" ht="15.75" customHeight="1" s="16">
+      <c r="A300" s="18" t="inlineStr">
+        <is>
+          <t>CHEIROSA 40</t>
+        </is>
+      </c>
+      <c r="B300" s="18" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="C300" s="18" t="inlineStr">
+        <is>
+          <t>Body Splash Inspiração</t>
+        </is>
+      </c>
+      <c r="D300" s="18" t="inlineStr">
+        <is>
+          <t>SOL DE JANEIRO</t>
+        </is>
+      </c>
+      <c r="E300" s="19" t="inlineStr">
+        <is>
+          <t>Floral Frutado</t>
+        </is>
+      </c>
+      <c r="F300" s="18" t="inlineStr">
+        <is>
+          <t>Body splash de inspiração (não é contratipo) · ordem na caixinha: 1 · família pesquisada pelo Claude</t>
+        </is>
+      </c>
+    </row>
+    <row r="301" ht="15.75" customHeight="1" s="16">
+      <c r="A301" s="18" t="inlineStr">
+        <is>
+          <t>CHEIROSA 48</t>
+        </is>
+      </c>
+      <c r="B301" s="18" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="C301" s="18" t="inlineStr">
+        <is>
+          <t>Body Splash Inspiração</t>
+        </is>
+      </c>
+      <c r="D301" s="18" t="inlineStr">
+        <is>
+          <t>SOL DE JANEIRO</t>
+        </is>
+      </c>
+      <c r="E301" s="19" t="inlineStr">
+        <is>
+          <t>Floral Frutado</t>
+        </is>
+      </c>
+      <c r="F301" s="18" t="inlineStr">
+        <is>
+          <t>Body splash de inspiração (não é contratipo) · ordem na caixinha: 2 · família pesquisada pelo Claude</t>
+        </is>
+      </c>
+    </row>
+    <row r="302" ht="15.75" customHeight="1" s="16">
+      <c r="A302" s="18" t="inlineStr">
+        <is>
+          <t>CHEIROSA 59</t>
+        </is>
+      </c>
+      <c r="B302" s="18" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="C302" s="18" t="inlineStr">
+        <is>
+          <t>Body Splash Inspiração</t>
+        </is>
+      </c>
+      <c r="D302" s="18" t="inlineStr">
+        <is>
+          <t>SOL DE JANEIRO</t>
+        </is>
+      </c>
+      <c r="E302" s="19" t="inlineStr">
+        <is>
+          <t>Oriental Floral</t>
+        </is>
+      </c>
+      <c r="F302" s="18" t="inlineStr">
+        <is>
+          <t>Body splash de inspiração (não é contratipo) · ordem na caixinha: 3 · família pesquisada pelo Claude</t>
+        </is>
+      </c>
+    </row>
+    <row r="303" ht="15.75" customHeight="1" s="16">
+      <c r="A303" s="18" t="inlineStr">
+        <is>
+          <t>CHEIROSA 62</t>
+        </is>
+      </c>
+      <c r="B303" s="18" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="C303" s="18" t="inlineStr">
+        <is>
+          <t>Body Splash Inspiração</t>
+        </is>
+      </c>
+      <c r="D303" s="18" t="inlineStr">
+        <is>
+          <t>SOL DE JANEIRO</t>
+        </is>
+      </c>
+      <c r="E303" s="19" t="inlineStr">
+        <is>
+          <t>Gourmand</t>
+        </is>
+      </c>
+      <c r="F303" s="18" t="inlineStr">
+        <is>
+          <t>Body splash de inspiração (não é contratipo) · ordem na caixinha: 4 · família pesquisada pelo Claude</t>
+        </is>
+      </c>
+    </row>
+    <row r="304" ht="15.75" customHeight="1" s="16">
+      <c r="A304" s="18" t="inlineStr">
+        <is>
+          <t>CHEIROSA 68</t>
+        </is>
+      </c>
+      <c r="B304" s="18" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="C304" s="18" t="inlineStr">
+        <is>
+          <t>Body Splash Inspiração</t>
+        </is>
+      </c>
+      <c r="D304" s="18" t="inlineStr">
+        <is>
+          <t>SOL DE JANEIRO</t>
+        </is>
+      </c>
+      <c r="E304" s="19" t="inlineStr">
+        <is>
+          <t>Floral Frutado</t>
+        </is>
+      </c>
+      <c r="F304" s="18" t="inlineStr">
+        <is>
+          <t>Body splash de inspiração (não é contratipo) · ordem na caixinha: 5 · família pesquisada pelo Claude</t>
+        </is>
+      </c>
+    </row>
+    <row r="305" ht="15.75" customHeight="1" s="16">
+      <c r="A305" s="18" t="inlineStr">
+        <is>
+          <t>DELEITE</t>
+        </is>
+      </c>
+      <c r="B305" s="18" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="C305" s="18" t="inlineStr">
+        <is>
+          <t>Body Splash Inspiração</t>
+        </is>
+      </c>
+      <c r="D305" s="18" t="inlineStr">
+        <is>
+          <t>O BOTICÁRIO</t>
+        </is>
+      </c>
+      <c r="E305" s="19" t="inlineStr">
+        <is>
+          <t>Gourmand</t>
+        </is>
+      </c>
+      <c r="F305" s="18" t="inlineStr">
+        <is>
+          <t>Body splash de inspiração (não é contratipo) · ordem na caixinha: 6 · família pesquisada pelo Claude</t>
+        </is>
+      </c>
+    </row>
+    <row r="306" ht="15.75" customHeight="1" s="16">
+      <c r="A306" s="18" t="inlineStr">
+        <is>
+          <t>GLAMOUR</t>
+        </is>
+      </c>
+      <c r="B306" s="18" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="C306" s="18" t="inlineStr">
+        <is>
+          <t>Body Splash Inspiração</t>
+        </is>
+      </c>
+      <c r="D306" s="18" t="inlineStr">
+        <is>
+          <t>O BOTICÁRIO</t>
+        </is>
+      </c>
+      <c r="E306" s="19" t="inlineStr">
+        <is>
+          <t>Oriental Floral</t>
+        </is>
+      </c>
+      <c r="F306" s="18" t="inlineStr">
+        <is>
+          <t>Body splash de inspiração · ordem na caixinha: 7 · inspirado no Glamour clássico do O Boticário (mandarina, ameixa, jasmim, lírio-do-vale, sândalo, baunilha)</t>
+        </is>
+      </c>
+    </row>
+    <row r="307" ht="15.75" customHeight="1" s="16">
+      <c r="A307" s="18" t="inlineStr">
+        <is>
+          <t>SOL DE CAJU</t>
+        </is>
+      </c>
+      <c r="B307" s="18" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="C307" s="18" t="inlineStr">
+        <is>
+          <t>Body Splash Inspiração</t>
+        </is>
+      </c>
+      <c r="D307" s="18" t="inlineStr">
+        <is>
+          <t>PHEBO</t>
+        </is>
+      </c>
+      <c r="E307" s="19" t="inlineStr">
+        <is>
+          <t>Frutado</t>
+        </is>
+      </c>
+      <c r="F307" s="18" t="inlineStr">
+        <is>
+          <t>Body splash de inspiração (não é contratipo) · ordem na caixinha: 8 · família pesquisada pelo Claude · inspirado em Isolda Cajueiro (Phebo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="308" ht="15.75" customHeight="1" s="16">
+      <c r="A308" s="18" t="inlineStr">
+        <is>
+          <t>ALGODÃO</t>
+        </is>
+      </c>
+      <c r="B308" s="18" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="C308" s="18" t="inlineStr">
+        <is>
+          <t>Body Splash Inspiração</t>
+        </is>
+      </c>
+      <c r="D308" s="18" t="inlineStr">
+        <is>
+          <t>NATURA</t>
+        </is>
+      </c>
+      <c r="E308" s="20" t="inlineStr">
+        <is>
+          <t>Floral Almiscarado</t>
+        </is>
+      </c>
+      <c r="F308" s="18" t="inlineStr">
+        <is>
+          <t>Body splash de inspiração · Big: Floral Aldeídico (aldeídos, íris, musk)</t>
+        </is>
+      </c>
+    </row>
+    <row r="309" ht="15.75" customHeight="1" s="16">
+      <c r="A309" s="18" t="inlineStr">
+        <is>
+          <t>BEBÊ NATURE</t>
+        </is>
+      </c>
+      <c r="B309" s="18" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="C309" s="18" t="inlineStr">
+        <is>
+          <t>Body Splash Inspiração</t>
+        </is>
+      </c>
+      <c r="D309" s="18" t="inlineStr">
+        <is>
+          <t>NATURA</t>
+        </is>
+      </c>
+      <c r="E309" s="20" t="inlineStr">
+        <is>
+          <t>Floral Amadeirado Almiscarado</t>
+        </is>
+      </c>
+      <c r="F309" s="18" t="inlineStr">
+        <is>
+          <t>Body splash de inspiração · Inspirado em Mamãe e Bebê; família do site da Big</t>
+        </is>
+      </c>
+    </row>
+    <row r="310" ht="15.75" customHeight="1" s="16">
+      <c r="A310" s="18" t="inlineStr">
+        <is>
+          <t>BARE VANILLA</t>
+        </is>
+      </c>
+      <c r="B310" s="18" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="C310" s="18" t="inlineStr">
+        <is>
+          <t>Body Splash Inspiração</t>
+        </is>
+      </c>
+      <c r="D310" s="18" t="inlineStr">
+        <is>
+          <t>VICTORIA'S SECRET</t>
+        </is>
+      </c>
+      <c r="E310" s="20" t="inlineStr">
+        <is>
+          <t>Oriental Baunilha</t>
+        </is>
+      </c>
+      <c r="F310" s="18" t="inlineStr">
+        <is>
+          <t>Body splash de inspiração · Big: Oriental Gourmand</t>
+        </is>
+      </c>
+    </row>
+    <row r="311" ht="15.75" customHeight="1" s="16">
+      <c r="A311" s="18" t="inlineStr">
+        <is>
+          <t>BIG BOSS</t>
+        </is>
+      </c>
+      <c r="B311" s="18" t="inlineStr">
+        <is>
+          <t>MASCULINO</t>
+        </is>
+      </c>
+      <c r="C311" s="18" t="inlineStr">
+        <is>
+          <t>Body Splash Inspiração</t>
+        </is>
+      </c>
+      <c r="D311" s="18" t="inlineStr">
+        <is>
+          <t>HUGO BOSS</t>
+        </is>
+      </c>
+      <c r="E311" s="19" t="inlineStr">
+        <is>
+          <t>Amadeirado Especiado</t>
+        </is>
+      </c>
+      <c r="F311" s="18" t="inlineStr">
+        <is>
+          <t>Body splash de inspiração · Inspirado em Boss Bottled</t>
+        </is>
+      </c>
+    </row>
+    <row r="312" ht="15.75" customHeight="1" s="16">
+      <c r="A312" s="18" t="inlineStr">
+        <is>
+          <t>COCONUT MILK AND ROSE</t>
+        </is>
+      </c>
+      <c r="B312" s="18" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="C312" s="18" t="inlineStr">
+        <is>
+          <t>Body Splash Inspiração</t>
+        </is>
+      </c>
+      <c r="D312" s="18" t="inlineStr">
+        <is>
+          <t>VICTORIA'S SECRET</t>
+        </is>
+      </c>
+      <c r="E312" s="20" t="inlineStr">
+        <is>
+          <t>Floral Gourmand</t>
+        </is>
+      </c>
+      <c r="F312" s="18" t="inlineStr">
+        <is>
+          <t>Body splash de inspiração · Big: Floral Frutado Gourmet</t>
+        </is>
+      </c>
+    </row>
+    <row r="313" ht="15.75" customHeight="1" s="16">
+      <c r="A313" s="18" t="inlineStr">
+        <is>
+          <t>COCONUT PASSION</t>
+        </is>
+      </c>
+      <c r="B313" s="18" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="C313" s="18" t="inlineStr">
+        <is>
+          <t>Body Splash Inspiração</t>
+        </is>
+      </c>
+      <c r="D313" s="18" t="inlineStr">
+        <is>
+          <t>VICTORIA'S SECRET</t>
+        </is>
+      </c>
+      <c r="E313" s="20" t="inlineStr">
+        <is>
+          <t>Gourmand</t>
+        </is>
+      </c>
+      <c r="F313" s="18" t="inlineStr">
+        <is>
+          <t>Body splash de inspiração · Big: Floral Frutado Gourmet (oriental)</t>
+        </is>
+      </c>
+    </row>
+    <row r="314" ht="15.75" customHeight="1" s="16">
+      <c r="A314" s="18" t="inlineStr">
+        <is>
+          <t>JOHN FRAGRANCE</t>
+        </is>
+      </c>
+      <c r="B314" s="18" t="inlineStr">
+        <is>
+          <t>MASCULINO</t>
+        </is>
+      </c>
+      <c r="C314" s="18" t="inlineStr">
+        <is>
+          <t>Body Splash Inspiração</t>
+        </is>
+      </c>
+      <c r="D314" s="18" t="inlineStr">
+        <is>
+          <t>JOHN JOHN</t>
+        </is>
+      </c>
+      <c r="E314" s="19" t="inlineStr">
+        <is>
+          <t>Amadeirado Aromático</t>
+        </is>
+      </c>
+      <c r="F314" s="18" t="inlineStr">
+        <is>
+          <t>Body splash de inspiração · Notas: limão, maçã, lavanda, vetiver, musk, baunilha</t>
+        </is>
+      </c>
+    </row>
+    <row r="315" ht="15.75" customHeight="1" s="16">
+      <c r="A315" s="18" t="inlineStr">
+        <is>
+          <t>LOVE SPELL</t>
+        </is>
+      </c>
+      <c r="B315" s="18" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="C315" s="18" t="inlineStr">
+        <is>
+          <t>Body Splash Inspiração</t>
+        </is>
+      </c>
+      <c r="D315" s="18" t="inlineStr">
+        <is>
+          <t>VICTORIA'S SECRET</t>
+        </is>
+      </c>
+      <c r="E315" s="20" t="inlineStr">
+        <is>
+          <t>Floral Frutado</t>
+        </is>
+      </c>
+      <c r="F315" s="18" t="inlineStr">
+        <is>
+          <t>Body splash de inspiração · Família do site da Big</t>
+        </is>
+      </c>
+    </row>
+    <row r="316" ht="15.75" customHeight="1" s="16">
+      <c r="A316" s="18" t="inlineStr">
+        <is>
+          <t>MACADÂMIA</t>
+        </is>
+      </c>
+      <c r="B316" s="18" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="C316" s="18" t="inlineStr">
+        <is>
+          <t>Body Splash Inspiração</t>
+        </is>
+      </c>
+      <c r="D316" s="18" t="inlineStr">
+        <is>
+          <t>NATURA</t>
+        </is>
+      </c>
+      <c r="E316" s="19" t="inlineStr">
+        <is>
+          <t>Floral Amadeirado</t>
+        </is>
+      </c>
+      <c r="F316" s="18" t="inlineStr">
+        <is>
+          <t>Body splash de inspiração · Notas: abacaxi, peônia, violeta, macadâmia, sândalo, musk</t>
+        </is>
+      </c>
+    </row>
+    <row r="317" ht="15.75" customHeight="1" s="16">
+      <c r="A317" s="18" t="inlineStr">
+        <is>
+          <t>PERFUME DA PRINCESA</t>
+        </is>
+      </c>
+      <c r="B317" s="18" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="C317" s="18" t="inlineStr">
+        <is>
+          <t>Body Splash Inspiração</t>
+        </is>
+      </c>
+      <c r="D317" s="18" t="inlineStr">
+        <is>
+          <t>CRIAÇÃO EXCLUSIVA</t>
+        </is>
+      </c>
+      <c r="E317" s="20" t="inlineStr">
+        <is>
+          <t>Floral Gourmand</t>
+        </is>
+      </c>
+      <c r="F317" s="18" t="inlineStr">
+        <is>
+          <t>Body splash de inspiração · Sem inspiração; família do site da Big</t>
+        </is>
+      </c>
+    </row>
+    <row r="318" ht="15.75" customHeight="1" s="16">
+      <c r="A318" s="18" t="inlineStr">
+        <is>
+          <t>PERFUME DA RAINHA</t>
+        </is>
+      </c>
+      <c r="B318" s="18" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="C318" s="18" t="inlineStr">
+        <is>
+          <t>Body Splash Inspiração</t>
+        </is>
+      </c>
+      <c r="D318" s="18" t="inlineStr">
+        <is>
+          <t>CRIAÇÃO EXCLUSIVA</t>
+        </is>
+      </c>
+      <c r="E318" s="20" t="inlineStr">
+        <is>
+          <t>Floral</t>
+        </is>
+      </c>
+      <c r="F318" s="18" t="inlineStr">
+        <is>
+          <t>Body splash de inspiração · Sem inspiração; família do site da Big</t>
+        </is>
+      </c>
+    </row>
+    <row r="319" ht="15.75" customHeight="1" s="16">
+      <c r="A319" s="18" t="inlineStr">
+        <is>
+          <t>PIMENTA ROSA</t>
+        </is>
+      </c>
+      <c r="B319" s="18" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="C319" s="18" t="inlineStr">
+        <is>
+          <t>Body Splash Inspiração</t>
+        </is>
+      </c>
+      <c r="D319" s="18" t="inlineStr">
+        <is>
+          <t>CRIAÇÃO EXCLUSIVA</t>
+        </is>
+      </c>
+      <c r="E319" s="20" t="inlineStr">
+        <is>
+          <t>Chipre Frutado</t>
+        </is>
+      </c>
+      <c r="F319" s="18" t="inlineStr">
+        <is>
+          <t>Body splash de inspiração · Sem inspiração; família do site da Big</t>
+        </is>
+      </c>
+    </row>
+    <row r="320" ht="15.75" customHeight="1" s="16">
+      <c r="A320" s="18" t="inlineStr">
+        <is>
+          <t>PRIPRIOCA</t>
+        </is>
+      </c>
+      <c r="B320" s="18" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="C320" s="18" t="inlineStr">
+        <is>
+          <t>Body Splash Inspiração</t>
+        </is>
+      </c>
+      <c r="D320" s="18" t="inlineStr">
+        <is>
+          <t>NATURA</t>
+        </is>
+      </c>
+      <c r="E320" s="20" t="inlineStr">
+        <is>
+          <t>Floral Aromático</t>
+        </is>
+      </c>
+      <c r="F320" s="18" t="inlineStr">
+        <is>
+          <t>Body splash de inspiração · Big: Floral Verde</t>
+        </is>
+      </c>
+    </row>
+    <row r="321" ht="15.75" customHeight="1" s="16">
+      <c r="A321" s="18" t="inlineStr">
+        <is>
+          <t>VELVET PETALS</t>
+        </is>
+      </c>
+      <c r="B321" s="18" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="C321" s="18" t="inlineStr">
+        <is>
+          <t>Body Splash Inspiração</t>
+        </is>
+      </c>
+      <c r="D321" s="18" t="inlineStr">
+        <is>
+          <t>VICTORIA'S SECRET</t>
+        </is>
+      </c>
+      <c r="E321" s="20" t="inlineStr">
+        <is>
+          <t>Floral Gourmand</t>
+        </is>
+      </c>
+      <c r="F321" s="18" t="inlineStr">
+        <is>
+          <t>Body splash de inspiração · Família do site da Big</t>
+        </is>
+      </c>
+    </row>
+    <row r="322" ht="15.75" customHeight="1" s="16">
+      <c r="A322" s="18" t="inlineStr">
+        <is>
+          <t>AMBER ROMANCE</t>
+        </is>
+      </c>
+      <c r="B322" s="18" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="C322" s="18" t="inlineStr">
+        <is>
+          <t>Body Splash Inspiração</t>
+        </is>
+      </c>
+      <c r="D322" s="18" t="inlineStr">
+        <is>
+          <t>VICTORIA'S SECRET</t>
+        </is>
+      </c>
+      <c r="E322" s="20" t="inlineStr">
+        <is>
+          <t>Oriental Baunilha</t>
+        </is>
+      </c>
+      <c r="F322" s="18" t="inlineStr">
+        <is>
+          <t>Body splash de inspiração · Big: Oriental Gourmand (açúcar, jasmim, sândalo, baunilha)</t>
+        </is>
+      </c>
+    </row>
+    <row r="323" ht="15.75" customHeight="1" s="16">
+      <c r="A323" s="18" t="inlineStr">
+        <is>
+          <t>GIOVANINHA</t>
+        </is>
+      </c>
+      <c r="B323" s="18" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="C323" s="18" t="inlineStr">
+        <is>
+          <t>Body Splash Inspiração</t>
+        </is>
+      </c>
+      <c r="D323" s="18" t="inlineStr">
+        <is>
+          <t>GIOVANNA BABY</t>
+        </is>
+      </c>
+      <c r="E323" s="20" t="inlineStr">
+        <is>
+          <t>Floral Aromático</t>
+        </is>
+      </c>
+      <c r="F323" s="18" t="inlineStr">
+        <is>
+          <t>Body splash de inspiração · Inspirado em Giovanna Baby Classic; família do site da Big</t>
+        </is>
+      </c>
+    </row>
+    <row r="324" ht="15.75" customHeight="1" s="16">
+      <c r="A324" s="18" t="inlineStr">
+        <is>
+          <t>BABY JOHN</t>
+        </is>
+      </c>
+      <c r="B324" s="18" t="inlineStr">
+        <is>
+          <t>FEMININO</t>
+        </is>
+      </c>
+      <c r="C324" s="18" t="inlineStr">
+        <is>
+          <t>Body Splash Inspiração</t>
+        </is>
+      </c>
+      <c r="D324" s="18" t="inlineStr">
+        <is>
+          <t>JOHNSON'S BABY</t>
+        </is>
+      </c>
+      <c r="E324" s="20" t="inlineStr">
+        <is>
+          <t>Floral Aromático</t>
+        </is>
+      </c>
+      <c r="F324" s="18" t="inlineStr">
+        <is>
+          <t>Body splash de inspiração · Inspirado na colônia clássica Johnson's Baby; Big: Aromática Verde</t>
+        </is>
+      </c>
+    </row>
     <row r="325" ht="15.75" customHeight="1" s="16"/>
     <row r="326" ht="15.75" customHeight="1" s="16"/>
     <row r="327" ht="15.75" customHeight="1" s="16"/>
@@ -10707,7 +11490,7 @@
     <row r="999" ht="15.75" customHeight="1" s="16"/>
     <row r="1000" ht="15.75" customHeight="1" s="16"/>
   </sheetData>
-  <autoFilter ref="$A$1:$F$299">
+  <autoFilter ref="A1:F324">
     <filterColumn colId="1" hiddenButton="0" showButton="1">
       <filters>
         <filter val="FEMININO"/>

</xml_diff>

<commit_message>
Planilha: família do The Blend Bourbon confirmada
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/arquivos/Fragrâncias Alquimikamente - FINAL.xlsx
+++ b/arquivos/Fragrâncias Alquimikamente - FINAL.xlsx
@@ -9412,14 +9412,14 @@
           <t>O BOTICÁRIO</t>
         </is>
       </c>
-      <c r="E280" s="23" t="inlineStr">
+      <c r="E280" s="21" t="inlineStr">
         <is>
           <t>Oriental Especiado</t>
         </is>
       </c>
       <c r="F280" s="14" t="inlineStr">
         <is>
-          <t>Nova (13/10) · vale conferir: fornecedor tem 'O Nobre Bourbon' (Oriental Especiada)</t>
+          <t>Nova (13/10) · família do site do fornecedor (O Nobre Bourbon, confirmado pela Lívia)</t>
         </is>
       </c>
     </row>

</xml_diff>